<commit_message>
Introduction TU MV Cas 03 et 03b
</commit_message>
<xml_diff>
--- a/Manuel Validation/CAS S02/Cas S02B.xlsx
+++ b/Manuel Validation/CAS S02/Cas S02B.xlsx
@@ -527,7 +527,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="0.00000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -808,7 +808,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -962,7 +962,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -974,7 +974,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -994,6 +994,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2196,8 +2199,8 @@
         <v>86</v>
       </c>
       <c r="E56" s="61">
-        <f>hw*tw*FyW/SQRT(3)/GammaM0/1000</f>
-        <v>2428.1702749917972</v>
+        <f>hw*tw*FyW/SQRT(3)/GammaM0/1000*Eta</f>
+        <v>2913.8043299901565</v>
       </c>
       <c r="F56" t="s">
         <v>13</v>
@@ -2233,7 +2236,7 @@
       </c>
       <c r="E58" s="60">
         <f>VEd_U1/VRd</f>
-        <v>0.15764957010739009</v>
+        <v>0.13137464175615843</v>
       </c>
       <c r="M58" s="3" t="s">
         <v>26</v>
@@ -2252,7 +2255,7 @@
       </c>
       <c r="E59" s="60">
         <f>VEd_U2/VRd</f>
-        <v>0.13096280902338048</v>
+        <v>0.1091356741861504</v>
       </c>
       <c r="M59" s="3"/>
     </row>
@@ -2262,7 +2265,7 @@
       </c>
       <c r="E60" s="75">
         <f>MAX(E58:E59)</f>
-        <v>0.15764957010739009</v>
+        <v>0.13137464175615843</v>
       </c>
       <c r="M60" s="3" t="s">
         <v>115</v>
@@ -2468,7 +2471,7 @@
       <c r="D76" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E76" s="75">
+      <c r="E76" s="81">
         <f>MAX(E74:E75)</f>
         <v>0.21474822331883595</v>
       </c>

</xml_diff>